<commit_message>
feat: add atomic capability runtime and comprehensive benchmark
</commit_message>
<xml_diff>
--- a/tests/agent_contract/data/H1_date_ambiguity.xlsx
+++ b/tests/agent_contract/data/H1_date_ambiguity.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,57 +413,79 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E129"/>
+  <dimension ref="A1:E149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n"/>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>订单号</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>订单日期</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>客户</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>金额</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>月份</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>订单号</t>
+          <t>O20001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>订单日期</t>
+          <t>2024-01-21</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>客户</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>金额</t>
-        </is>
+          <t>客户1112</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2767</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>月份</t>
+          <t>1月</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>O20001</t>
+          <t>O20002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2024/01/04</t>
+          <t>01/18/2024</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>客户1730</t>
+          <t>客户1884</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3974</v>
+        <v>3971</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -478,21 +496,21 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>O20002</t>
+          <t>O20003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>18/01/2024</t>
+          <t>2024-01-09</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>客户1440</t>
+          <t>客户1411</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1609</v>
+        <v>2065</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -503,21 +521,21 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>O20003</t>
+          <t>O20004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10/01/2024</t>
+          <t>01/03/2024</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>客户1981</t>
+          <t>客户1676</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1680</v>
+        <v>2177</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -528,21 +546,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>O20004</t>
+          <t>O20005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2024-01-17</t>
+          <t>2024-01-10</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>客户1761</t>
+          <t>客户1754</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2032</v>
+        <v>1739</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -553,21 +571,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>O20005</t>
+          <t>O20006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2024-01-11</t>
+          <t>2024-01-20</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>客户1877</t>
+          <t>客户1118</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3472</v>
+        <v>1519</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -578,21 +596,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>O20006</t>
+          <t>O20007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2024-01-13</t>
+          <t>01/16/2024</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>客户1380</t>
+          <t>客户1954</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3454</v>
+        <v>1646</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -603,21 +621,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>O20007</t>
+          <t>O20008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>01/01/2024</t>
+          <t>2024-01-20</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>客户1211</t>
+          <t>客户1279</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1754</v>
+        <v>1507</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -628,21 +646,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>O20008</t>
+          <t>O20009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>01/23/2024</t>
+          <t>09/01/2024</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>客户1418</t>
+          <t>客户1847</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10025</v>
+        <v>1533</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -653,171 +671,171 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>O20009</t>
+          <t>O20010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>02/02/2024</t>
+          <t>2024-01-10</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>客户1529</t>
+          <t>客户1665</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3892</v>
+        <v>1557</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2月</t>
+          <t>1月</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>O20010</t>
+          <t>O20011</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>02/28/2024</t>
+          <t>2024/01/28</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>客户1102</t>
+          <t>客户1545</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1831</v>
+        <v>1516</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2月</t>
+          <t>1月</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>O20011</t>
+          <t>O20012</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>26/02/2024</t>
+          <t>2024/01/09</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>客户1165</t>
+          <t>客户1430</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2651</v>
+        <v>1500</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2月</t>
+          <t>1月</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>O20012</t>
+          <t>O20013</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2024-02-07</t>
+          <t>2024-01-14</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>客户1755</t>
+          <t>客户1789</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3453</v>
+        <v>1503</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2月</t>
+          <t>1月</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>O20013</t>
+          <t>O20014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2024/02/16</t>
+          <t>2024-01-06</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>客户1706</t>
+          <t>客户1406</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3636</v>
+        <v>1500</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2月</t>
+          <t>1月</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>O20014</t>
+          <t>O20015</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>11/02/2024</t>
+          <t>09/01/2024</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>客户1494</t>
+          <t>客户1213</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>3932</v>
+        <v>1500</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2月</t>
+          <t>1月</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>O20015</t>
+          <t>O20016</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>21/02/2024</t>
+          <t>02/14/2024</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>客户1315</t>
+          <t>客户1485</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3638</v>
+        <v>2931</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -828,21 +846,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>O20016</t>
+          <t>O20017</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2024-02-04</t>
+          <t>02/14/2024</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>客户1734</t>
+          <t>客户1150</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1589</v>
+        <v>3363</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -853,21 +871,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>O20017</t>
+          <t>O20018</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2024/02/13</t>
+          <t>05/02/2024</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>客户1782</t>
+          <t>客户1206</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3442</v>
+        <v>3072</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -878,21 +896,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>O20018</t>
+          <t>O20019</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2024/02/11</t>
+          <t>02/09/2024</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>客户1536</t>
+          <t>客户1047</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3936</v>
+        <v>2806</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -903,121 +921,121 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>O20019</t>
+          <t>O20020</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>08/03/2024</t>
+          <t>2024-02-27</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>客户1575</t>
+          <t>客户1852</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1611</v>
+        <v>3974</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>3月</t>
+          <t>2月</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>O20020</t>
+          <t>O20021</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2024/03/06</t>
+          <t>2024-02-06</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>客户1930</t>
+          <t>客户1599</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>3990</v>
+        <v>2491</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>3月</t>
+          <t>2月</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>O20021</t>
+          <t>O20022</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2024-03-12</t>
+          <t>2024-02-11</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>客户1949</t>
+          <t>客户1563</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2170</v>
+        <v>1737</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3月</t>
+          <t>2月</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>O20022</t>
+          <t>O20023</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2024-03-13</t>
+          <t>02/06/2024</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>客户1378</t>
+          <t>客户1930</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3519</v>
+        <v>11626</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>3月</t>
+          <t>2月</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>O20023</t>
+          <t>O20024</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>03/06/2024</t>
+          <t>03/11/2024</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>客户1574</t>
+          <t>客户1355</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2750</v>
+        <v>2972</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1028,21 +1046,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>O20024</t>
+          <t>O20025</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2024-03-13</t>
+          <t>2024/03/07</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>客户1867</t>
+          <t>客户1207</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1821</v>
+        <v>2815</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1053,21 +1071,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>O20025</t>
+          <t>O20026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>07/03/2024</t>
+          <t>03/01/2024</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>客户1106</t>
+          <t>客户1958</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2374</v>
+        <v>3580</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1078,21 +1096,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>O20026</t>
+          <t>O20027</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2024/03/19</t>
+          <t>2024/03/15</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>客户1396</t>
+          <t>客户1910</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3384</v>
+        <v>3812</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1103,21 +1121,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>O20027</t>
+          <t>O20028</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>05/03/2024</t>
+          <t>2024-03-19</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>客户1770</t>
+          <t>客户1653</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2564</v>
+        <v>2639</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1128,21 +1146,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>O20028</t>
+          <t>O20029</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2024-03-13</t>
+          <t>2024/03/21</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>客户1324</t>
+          <t>客户1757</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2471</v>
+        <v>2624</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1153,21 +1171,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>O20029</t>
+          <t>O20030</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2024-03-08</t>
+          <t>2024-03-16</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>客户1690</t>
+          <t>客户1768</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2914</v>
+        <v>3155</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1178,21 +1196,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>O20030</t>
+          <t>O20031</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>26/03/2024</t>
+          <t>2024/03/25</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>客户1976</t>
+          <t>客户1930</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2015</v>
+        <v>13403</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1203,71 +1221,71 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>O20031</t>
+          <t>O20032</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2024-03-17</t>
+          <t>04/04/2024</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>客户1934</t>
+          <t>客户1783</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1761</v>
+        <v>2424</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>3月</t>
+          <t>4月</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>O20032</t>
+          <t>O20033</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2024/03/26</t>
+          <t>2024-04-21</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>客户1342</t>
+          <t>客户1092</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1656</v>
+        <v>2575</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>3月</t>
+          <t>4月</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>O20033</t>
+          <t>O20034</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>07/04/2024</t>
+          <t>2024/04/19</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>客户1204</t>
+          <t>客户1841</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>2472</v>
+        <v>2954</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1278,21 +1296,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>O20034</t>
+          <t>O20035</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2024-04-07</t>
+          <t>24/04/2024</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>客户1920</t>
+          <t>客户1076</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>3675</v>
+        <v>3897</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1303,21 +1321,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>O20035</t>
+          <t>O20036</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>04/07/2024</t>
+          <t>04/24/2024</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>客户1270</t>
+          <t>客户1965</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>3013</v>
+        <v>2445</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1328,21 +1346,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>O20036</t>
+          <t>O20037</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>04/20/2024</t>
+          <t>2024-04-26</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>客户1719</t>
+          <t>客户1466</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>2222</v>
+        <v>1961</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1353,21 +1371,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>O20037</t>
+          <t>O20038</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2024-04-08</t>
+          <t>2024-04-25</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>客户1314</t>
+          <t>客户1594</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1843</v>
+        <v>1667</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1378,21 +1396,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>O20038</t>
+          <t>O20039</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2024-04-27</t>
+          <t>2024/04/10</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>客户1809</t>
+          <t>客户1652</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>3061</v>
+        <v>1694</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1403,21 +1421,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>O20039</t>
+          <t>O20040</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2024-04-17</t>
+          <t>18/04/2024</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>客户1055</t>
+          <t>客户1086</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>2767</v>
+        <v>3414</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1428,21 +1446,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>O20040</t>
+          <t>O20041</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>04/19/2024</t>
+          <t>2024/04/09</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>客户1376</t>
+          <t>客户1276</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>3614</v>
+        <v>2650</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1453,21 +1471,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>O20041</t>
+          <t>O20042</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2024-04-01</t>
+          <t>2024-04-24</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>客户1464</t>
+          <t>客户1223</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>3046</v>
+        <v>2290</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1478,21 +1496,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>O20042</t>
+          <t>O20043</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2024-04-03</t>
+          <t>16/04/2024</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>客户1403</t>
+          <t>客户1597</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>12287</v>
+        <v>2159</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1503,96 +1521,96 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>O20043</t>
+          <t>O20044</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>05/24/2024</t>
+          <t>2024/04/16</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>客户1401</t>
+          <t>客户1691</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1725</v>
+        <v>3276</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>5月</t>
+          <t>4月</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>O20044</t>
+          <t>O20045</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2024-05-03</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>客户1810</t>
+          <t>客户1248</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>3804</v>
+        <v>2741</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>5月</t>
+          <t>4月</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>O20045</t>
+          <t>O20046</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>05/19/2024</t>
+          <t>20/04/2024</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>客户1188</t>
+          <t>客户1714</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1985</v>
+        <v>1853</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>5月</t>
+          <t>4月</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>O20046</t>
+          <t>O20047</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>05/13/2024</t>
+          <t>05/03/2024</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>客户1256</t>
+          <t>客户1920</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>3516</v>
+        <v>2552</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1603,21 +1621,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>O20047</t>
+          <t>O20048</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2024-05-01</t>
+          <t>17/05/2024</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>客户1786</t>
+          <t>客户1436</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>3191</v>
+        <v>1789</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1628,21 +1646,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>O20048</t>
+          <t>O20049</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2024-05-13</t>
+          <t>05/20/2024</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>客户1476</t>
+          <t>客户1235</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1695</v>
+        <v>3266</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1653,21 +1671,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>O20049</t>
+          <t>O20050</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>05/27/2024</t>
+          <t>05/22/2024</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>客户1955</t>
+          <t>客户1598</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>3330</v>
+        <v>2015</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1678,21 +1696,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>O20050</t>
+          <t>O20051</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>15/05/2024</t>
+          <t>05/08/2024</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>客户1586</t>
+          <t>客户1520</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>2992</v>
+        <v>3071</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1703,21 +1721,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>O20051</t>
+          <t>O20052</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>05/15/2024</t>
+          <t>2024/05/11</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>客户1061</t>
+          <t>客户1621</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>3824</v>
+        <v>2439</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1728,21 +1746,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>O20052</t>
+          <t>O20053</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>17/05/2024</t>
+          <t>2024/05/14</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>客户1837</t>
+          <t>客户1923</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>2510</v>
+        <v>1629</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1753,21 +1771,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>O20053</t>
+          <t>O20054</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>05/03/2024</t>
+          <t>05/05/2024</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>客户1390</t>
+          <t>客户1101</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>1626</v>
+        <v>3005</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1778,21 +1796,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>O20054</t>
+          <t>O20055</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2024/05/10</t>
+          <t>2024-05-27</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>客户1895</t>
+          <t>客户1438</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>11802</v>
+        <v>1874</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1803,121 +1821,121 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>O20055</t>
+          <t>O20056</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2024-06-18</t>
+          <t>2024/05/11</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>客户1164</t>
+          <t>客户1083</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>3817</v>
+        <v>1556</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>6月</t>
+          <t>5月</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>O20056</t>
+          <t>O20057</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>06/27/2024</t>
+          <t>28/05/2024</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>客户1637</t>
+          <t>客户1083</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>2339</v>
+        <v>3637</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>6月</t>
+          <t>5月</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>O20057</t>
+          <t>O20058</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>06/20/2024</t>
+          <t>2024/05/05</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>客户1458</t>
+          <t>客户1846</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>2123</v>
+        <v>3335</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>6月</t>
+          <t>5月</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>O20058</t>
+          <t>O20059</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>26/06/2024</t>
+          <t>2024/05/19</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>客户1823</t>
+          <t>客户1652</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>2857</v>
+        <v>11832</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>6月</t>
+          <t>5月</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>O20059</t>
+          <t>O20060</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>16/06/2024</t>
+          <t>2024/06/10</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>客户1557</t>
+          <t>客户1780</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>1620</v>
+        <v>2314</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1928,21 +1946,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>O20060</t>
+          <t>O20061</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>06/27/2024</t>
+          <t>06/24/2024</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>客户1373</t>
+          <t>客户1523</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>1608</v>
+        <v>3074</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1953,21 +1971,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>O20061</t>
+          <t>O20062</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2024-06-18</t>
+          <t>2024-06-03</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>客户1174</t>
+          <t>客户1401</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1740</v>
+        <v>2672</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1978,21 +1996,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>O20062</t>
+          <t>O20063</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>06/21/2024</t>
+          <t>2024/06/04</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>客户1552</t>
+          <t>客户1516</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>2956</v>
+        <v>2788</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2003,21 +2021,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>O20063</t>
+          <t>O20064</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>01/06/2024</t>
+          <t>08/06/2024</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>客户1357</t>
+          <t>客户1404</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>3762</v>
+        <v>2619</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2028,21 +2046,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>O20064</t>
+          <t>O20065</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>06/15/2024</t>
+          <t>2024/06/27</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>客户1133</t>
+          <t>客户1276</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>22178</v>
+        <v>3243</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2053,171 +2071,171 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>O20065</t>
+          <t>O20066</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2024/07/25</t>
+          <t>2024/06/24</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>客户1877</t>
+          <t>客户1485</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>2313</v>
+        <v>1572</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>7月</t>
+          <t>6月</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>O20066</t>
+          <t>O20067</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>24/07/2024</t>
+          <t>19/06/2024</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>客户1301</t>
+          <t>客户1228</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>3511</v>
+        <v>2993</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>7月</t>
+          <t>6月</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>O20067</t>
+          <t>O20068</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2024/07/12</t>
+          <t>2024-06-10</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>客户1036</t>
+          <t>客户1740</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>2878</v>
+        <v>2160</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>7月</t>
+          <t>6月</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>O20068</t>
+          <t>O20069</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2024/07/28</t>
+          <t>06/02/2024</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>客户1170</t>
+          <t>客户1833</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>3362</v>
+        <v>2018</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>7月</t>
+          <t>6月</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>O20069</t>
+          <t>O20070</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2024-07-10</t>
+          <t>2024-06-04</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>客户1201</t>
+          <t>客户1033</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>2255</v>
+        <v>2103</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>7月</t>
+          <t>6月</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>O20070</t>
+          <t>O20071</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2024-07-19</t>
+          <t>2024/06/04</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>客户1690</t>
+          <t>客户1327</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>2852</v>
+        <v>17444</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>7月</t>
+          <t>6月</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>O20071</t>
+          <t>O20072</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>07/15/2024</t>
+          <t>2024-07-08</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>客户1364</t>
+          <t>客户1588</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>2167</v>
+        <v>2458</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2228,21 +2246,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>O20072</t>
+          <t>O20073</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2024/07/12</t>
+          <t>05/07/2024</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>客户1948</t>
+          <t>客户1455</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>28662</v>
+        <v>2333</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2253,1373 +2271,1873 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>O20073</t>
+          <t>O20074</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>14/08/2024</t>
+          <t>2024/07/09</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>客户1525</t>
+          <t>客户1698</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>1551</v>
+        <v>3201</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>8月</t>
+          <t>7月</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>O20074</t>
+          <t>O20075</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>07/08/2024</t>
+          <t>2024-07-10</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>客户1389</t>
+          <t>客户1654</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>1802</v>
+        <v>2737</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>8月</t>
+          <t>7月</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>O20075</t>
+          <t>O20076</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2024/08/28</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>客户1869</t>
+          <t>客户1991</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>3148</v>
+        <v>3726</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>8月</t>
+          <t>7月</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>O20076</t>
+          <t>O20077</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2024-08-14</t>
+          <t>07/05/2024</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>客户1411</t>
+          <t>客户1267</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>3025</v>
+        <v>3635</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>8月</t>
+          <t>7月</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>O20077</t>
+          <t>O20078</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2024/08/27</t>
+          <t>07/27/2024</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>客户1896</t>
+          <t>客户1841</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>3960</v>
+        <v>2729</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>8月</t>
+          <t>7月</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>O20078</t>
+          <t>O20079</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>08/02/2024</t>
+          <t>2024-07-21</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>客户1607</t>
+          <t>客户1631</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>3595</v>
+        <v>2112</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>8月</t>
+          <t>7月</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>O20079</t>
+          <t>O20080</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2024/08/15</t>
+          <t>07/24/2024</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>客户1428</t>
+          <t>客户1131</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>2866</v>
+        <v>3609</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>8月</t>
+          <t>7月</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>O20080</t>
+          <t>O20081</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2024-08-13</t>
+          <t>07/13/2024</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>客户1592</t>
+          <t>客户1030</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>3835</v>
+        <v>3051</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>8月</t>
+          <t>7月</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>O20081</t>
+          <t>O20082</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2024/08/06</t>
+          <t>23/07/2024</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>客户1718</t>
+          <t>客户1922</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>3865</v>
+        <v>3542</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>8月</t>
+          <t>7月</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>O20082</t>
+          <t>O20083</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2024/08/27</t>
+          <t>04/07/2024</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>客户1476</t>
+          <t>客户1248</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>24353</v>
+        <v>3959</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>8月</t>
+          <t>7月</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>O20083</t>
+          <t>O20084</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>08/09/2024</t>
+          <t>07/12/2024</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>客户1233</t>
+          <t>客户1610</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>1930</v>
+        <v>10908</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>9月</t>
+          <t>7月</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>O20084</t>
+          <t>O20085</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2024-09-25</t>
+          <t>08/05/2024</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>客户1262</t>
+          <t>客户1520</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>2958</v>
+        <v>3537</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>9月</t>
+          <t>8月</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>O20085</t>
+          <t>O20086</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>09/06/2024</t>
+          <t>11/08/2024</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>客户1160</t>
+          <t>客户1249</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>2796</v>
+        <v>2480</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>9月</t>
+          <t>8月</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>O20086</t>
+          <t>O20087</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2024/09/22</t>
+          <t>04/08/2024</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>客户1483</t>
+          <t>客户1316</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>3615</v>
+        <v>2203</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>9月</t>
+          <t>8月</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>O20087</t>
+          <t>O20088</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2024-09-06</t>
+          <t>2024/08/05</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>客户1793</t>
+          <t>客户1916</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>3806</v>
+        <v>2447</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>9月</t>
+          <t>8月</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>O20088</t>
+          <t>O20089</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2024-09-17</t>
+          <t>08/23/2024</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>客户1405</t>
+          <t>客户1932</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>3548</v>
+        <v>3952</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>9月</t>
+          <t>8月</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>O20089</t>
+          <t>O20090</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>24/09/2024</t>
+          <t>11/08/2024</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>客户1684</t>
+          <t>客户1941</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>1875</v>
+        <v>3598</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>9月</t>
+          <t>8月</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>O20090</t>
+          <t>O20091</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>28/09/2024</t>
+          <t>04/08/2024</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>客户1183</t>
+          <t>客户1461</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>3458</v>
+        <v>3923</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>9月</t>
+          <t>8月</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>O20091</t>
+          <t>O20092</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>09/19/2024</t>
+          <t>12/08/2024</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>客户1183</t>
+          <t>客户1241</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>31014</v>
+        <v>3724</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>9月</t>
+          <t>8月</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>O20092</t>
+          <t>O20093</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2024-10-27</t>
+          <t>23/08/2024</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>客户1037</t>
+          <t>客户1039</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>3967</v>
+        <v>2270</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>8月</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>O20093</t>
+          <t>O20094</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2024/10/13</t>
+          <t>2024-08-19</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>客户1138</t>
+          <t>客户1581</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>1737</v>
+        <v>3582</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>8月</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>O20094</t>
+          <t>O20095</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>10/17/2024</t>
+          <t>2024/08/25</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>客户1505</t>
+          <t>客户1971</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>1798</v>
+        <v>2959</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>8月</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>O20095</t>
+          <t>O20096</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>10/18/2024</t>
+          <t>08/13/2024</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>客户1188</t>
+          <t>客户1154</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>3673</v>
+        <v>2213</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>8月</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>O20096</t>
+          <t>O20097</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>04/10/2024</t>
+          <t>08/20/2024</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>客户1904</t>
+          <t>客户1263</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>2288</v>
+        <v>2248</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>8月</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>O20097</t>
+          <t>O20098</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>23/10/2024</t>
+          <t>08/09/2024</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>客户1403</t>
+          <t>客户1614</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>3855</v>
+        <v>12864</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>8月</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>O20098</t>
+          <t>O20099</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2024-10-10</t>
+          <t>28/09/2024</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>客户1475</t>
+          <t>客户1333</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>3189</v>
+        <v>1811</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>9月</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>O20099</t>
+          <t>O20100</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2024/10/19</t>
+          <t>2024-09-27</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>客户1694</t>
+          <t>客户1553</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>3364</v>
+        <v>2941</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>9月</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>O20100</t>
+          <t>O20101</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>09/10/2024</t>
+          <t>2024/09/28</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>客户1261</t>
+          <t>客户1303</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>2501</v>
+        <v>1667</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>9月</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>O20101</t>
+          <t>O20102</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2024-10-19</t>
+          <t>17/09/2024</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>客户1613</t>
+          <t>客户1905</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>3795</v>
+        <v>1539</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>9月</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>O20102</t>
+          <t>O20103</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>10/13/2024</t>
+          <t>2024-09-07</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>客户1366</t>
+          <t>客户1862</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>3240</v>
+        <v>3397</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>9月</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>O20103</t>
+          <t>O20104</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2024/10/17</t>
+          <t>09/21/2024</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>客户1022</t>
+          <t>客户1439</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>3705</v>
+        <v>3588</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>9月</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>O20104</t>
+          <t>O20105</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2024/10/26</t>
+          <t>09/20/2024</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>客户1554</t>
+          <t>客户1506</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>3763</v>
+        <v>3286</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>9月</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>O20105</t>
+          <t>O20106</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2024/10/03</t>
+          <t>09/11/2024</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>客户1484</t>
+          <t>客户1148</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>17125</v>
+        <v>3960</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>9月</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>O20106</t>
+          <t>O20107</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>02/11/2024</t>
+          <t>2024-09-19</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>客户1228</t>
+          <t>客户1223</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>3266</v>
+        <v>3317</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>9月</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>O20107</t>
+          <t>O20108</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2024-11-15</t>
+          <t>07/09/2024</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>客户1161</t>
+          <t>客户1907</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>3033</v>
+        <v>2807</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>9月</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>O20108</t>
+          <t>O20109</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2024-11-02</t>
+          <t>09/12/2024</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>客户1243</t>
+          <t>客户1486</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>3634</v>
+        <v>3499</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>9月</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>O20109</t>
+          <t>O20110</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2024/11/10</t>
+          <t>2024-09-05</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>客户1230</t>
+          <t>客户1437</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>3343</v>
+        <v>23188</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>9月</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>O20110</t>
+          <t>O20111</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>12/11/2024</t>
+          <t>25/10/2024</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>客户1670</t>
+          <t>客户1133</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>2751</v>
+        <v>1647</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>10月</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>O20111</t>
+          <t>O20112</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>24/11/2024</t>
+          <t>2024-10-25</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>客户1105</t>
+          <t>客户1458</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>3553</v>
+        <v>3362</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>10月</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>O20112</t>
+          <t>O20113</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>18/11/2024</t>
+          <t>2024/10/22</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>客户1188</t>
+          <t>客户1766</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>3700</v>
+        <v>3224</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>10月</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>O20113</t>
+          <t>O20114</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2024/11/09</t>
+          <t>2024/10/15</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>客户1293</t>
+          <t>客户1995</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>3264</v>
+        <v>1898</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>10月</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>O20114</t>
+          <t>O20115</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2024-11-15</t>
+          <t>10/15/2024</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>客户1894</t>
+          <t>客户1528</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>1673</v>
+        <v>1797</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>10月</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>O20115</t>
+          <t>O20116</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>01/11/2024</t>
+          <t>16/10/2024</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>客户1531</t>
+          <t>客户1978</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>2175</v>
+        <v>3375</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>10月</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>O20116</t>
+          <t>O20117</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2024/11/22</t>
+          <t>25/10/2024</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>客户1114</t>
+          <t>客户1602</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>1623</v>
+        <v>3886</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>10月</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>O20117</t>
+          <t>O20118</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>12/11/2024</t>
+          <t>2024-10-17</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>客户1440</t>
+          <t>客户1106</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>3451</v>
+        <v>3619</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>10月</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>O20118</t>
+          <t>O20119</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2024-11-25</t>
+          <t>2024-10-25</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>客户1045</t>
+          <t>客户1162</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>2401</v>
+        <v>2485</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>10月</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>O20119</t>
+          <t>O20120</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2024/11/02</t>
+          <t>2024-10-25</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>客户1773</t>
+          <t>客户1960</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>24133</v>
+        <v>3005</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>10月</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>O20120</t>
+          <t>O20121</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2024/12/08</t>
+          <t>2024/10/19</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>客户1720</t>
+          <t>客户1533</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>2762</v>
+        <v>2325</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>12月</t>
+          <t>10月</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>O20121</t>
+          <t>O20122</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>03/12/2024</t>
+          <t>2024-10-16</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>客户1246</t>
+          <t>客户1511</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>3430</v>
+        <v>3959</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>12月</t>
+          <t>10月</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>O20122</t>
+          <t>O20123</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>12/12/2024</t>
+          <t>03/10/2024</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>客户1850</t>
+          <t>客户1825</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>3815</v>
+        <v>23418</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>12月</t>
+          <t>10月</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>O20123</t>
+          <t>O20124</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>12/05/2024</t>
+          <t>11/14/2024</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>客户1728</t>
+          <t>客户1020</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>2836</v>
+        <v>3166</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>12月</t>
+          <t>11月</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>O20124</t>
+          <t>O20125</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>12/22/2024</t>
+          <t>2024/11/24</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>客户1628</t>
+          <t>客户1629</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>3335</v>
+        <v>3914</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>12月</t>
+          <t>11月</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>O20125</t>
+          <t>O20126</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2024/12/10</t>
+          <t>17/11/2024</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>客户1379</t>
+          <t>客户1300</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>2964</v>
+        <v>3552</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>12月</t>
+          <t>11月</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>O20126</t>
+          <t>O20127</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>28/12/2024</t>
+          <t>26/11/2024</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>客户1194</t>
+          <t>客户1455</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>3965</v>
+        <v>1691</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>12月</t>
+          <t>11月</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>O20127</t>
+          <t>O20128</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2024/12/23</t>
+          <t>2024/11/01</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>客户1709</t>
+          <t>客户1163</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>41893</v>
+        <v>2650</v>
       </c>
       <c r="E129" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>O20129</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2024-11-27</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>客户1664</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>3778</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>O20130</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>11/28/2024</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>客户1585</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>3920</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>O20131</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2024/11/08</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>客户1636</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>2089</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>O20132</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2024/11/08</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>客户1103</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>2118</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>O20133</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2024-11-25</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>客户1761</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>2968</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>O20134</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>15/11/2024</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>客户1714</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>3943</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>O20135</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>23/11/2024</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>客户1264</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>28211</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>O20136</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>2024-12-11</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>客户1164</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>1615</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>O20137</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>07/12/2024</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>客户1332</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>2394</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>O20138</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2024-12-02</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>客户1809</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>1879</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>O20139</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>2024/12/11</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>客户1687</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>1733</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>O20140</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>2024-12-01</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>客户1617</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>1906</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>O20141</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>12/05/2024</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>客户1270</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>2754</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>O20142</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>12/28/2024</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>客户1063</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>3672</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>O20143</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>2024/12/02</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>客户1137</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>1863</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>O20144</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>2024-12-22</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>客户1537</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>3366</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>O20145</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>2024-12-21</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>客户1776</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>3698</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>O20146</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>19/12/2024</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>客户1678</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>2753</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>O20147</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>12/06/2024</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>客户1345</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>3876</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>O20148</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>06/12/2024</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>客户1186</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>33491</v>
+      </c>
+      <c r="E149" t="inlineStr">
         <is>
           <t>12月</t>
         </is>

</xml_diff>